<commit_message>
Female masters bw were copy-pasted wrong; closes #1372
</commit_message>
<xml_diff>
--- a/owlcms/src/main/resources/agegroups/AgeGroups_2026-08.xlsx
+++ b/owlcms/src/main/resources/agegroups/AgeGroups_2026-08.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lamyj\git\owlcms4\owlcms\src\main\resources\agegroups\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\git\owlcms4\owlcms\src\main\resources\agegroups\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1ECBC620-182C-4E6B-AB96-D537D560B78A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF5165AA-CCEB-4741-A9A4-EF83D0272A6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AgeGroups" sheetId="1" r:id="rId1"/>
@@ -354,7 +354,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -377,7 +377,6 @@
     </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -980,28 +979,28 @@
       </c>
       <c r="M7" s="6"/>
       <c r="N7" s="6" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="O7" s="6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P7" s="6" t="s">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="Q7" s="6" t="s">
-        <v>15</v>
+        <v>37</v>
       </c>
       <c r="R7" s="6" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="S7" s="6" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="T7" s="6" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="U7" s="6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1032,28 +1031,28 @@
       </c>
       <c r="M8" s="6"/>
       <c r="N8" s="6" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="O8" s="6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P8" s="6" t="s">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="Q8" s="6" t="s">
-        <v>15</v>
+        <v>37</v>
       </c>
       <c r="R8" s="6" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="S8" s="6" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="T8" s="6" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="U8" s="6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1084,28 +1083,28 @@
       </c>
       <c r="M9" s="6"/>
       <c r="N9" s="6" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="O9" s="6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P9" s="6" t="s">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="Q9" s="6" t="s">
-        <v>15</v>
+        <v>37</v>
       </c>
       <c r="R9" s="6" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="S9" s="6" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="T9" s="6" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="U9" s="6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1133,28 +1132,28 @@
       </c>
       <c r="M10" s="6"/>
       <c r="N10" s="6" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="O10" s="6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P10" s="6" t="s">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="Q10" s="6" t="s">
-        <v>15</v>
+        <v>37</v>
       </c>
       <c r="R10" s="6" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="S10" s="6" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="T10" s="6" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="U10" s="6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1182,28 +1181,28 @@
       </c>
       <c r="M11" s="6"/>
       <c r="N11" s="6" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="O11" s="6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P11" s="6" t="s">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="Q11" s="6" t="s">
-        <v>15</v>
+        <v>37</v>
       </c>
       <c r="R11" s="6" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="S11" s="6" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="T11" s="6" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="U11" s="6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="12" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1234,28 +1233,28 @@
       </c>
       <c r="M12" s="6"/>
       <c r="N12" s="6" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="O12" s="6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P12" s="6" t="s">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="Q12" s="6" t="s">
-        <v>15</v>
+        <v>37</v>
       </c>
       <c r="R12" s="6" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="S12" s="6" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="T12" s="6" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="U12" s="6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="13" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1286,28 +1285,28 @@
       </c>
       <c r="M13" s="6"/>
       <c r="N13" s="6" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="O13" s="6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P13" s="6" t="s">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="Q13" s="6" t="s">
-        <v>15</v>
+        <v>37</v>
       </c>
       <c r="R13" s="6" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="S13" s="6" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="T13" s="6" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="U13" s="6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="14" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1338,28 +1337,28 @@
       </c>
       <c r="M14" s="6"/>
       <c r="N14" s="6" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="O14" s="6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P14" s="6" t="s">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="Q14" s="6" t="s">
-        <v>15</v>
+        <v>37</v>
       </c>
       <c r="R14" s="6" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="S14" s="6" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="T14" s="6" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="U14" s="6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1390,28 +1389,28 @@
       </c>
       <c r="M15" s="6"/>
       <c r="N15" s="6" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="O15" s="6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P15" s="6" t="s">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="Q15" s="6" t="s">
-        <v>15</v>
+        <v>37</v>
       </c>
       <c r="R15" s="6" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="S15" s="6" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="T15" s="6" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="U15" s="6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="16" spans="1:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1442,28 +1441,28 @@
       </c>
       <c r="M16" s="6"/>
       <c r="N16" s="6" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="O16" s="6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P16" s="6" t="s">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="Q16" s="6" t="s">
-        <v>15</v>
+        <v>37</v>
       </c>
       <c r="R16" s="6" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="S16" s="6" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="T16" s="6" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="U16" s="6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="17" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1494,28 +1493,28 @@
       </c>
       <c r="M17" s="6"/>
       <c r="N17" s="6" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="O17" s="6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P17" s="6" t="s">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="Q17" s="6" t="s">
-        <v>15</v>
+        <v>37</v>
       </c>
       <c r="R17" s="6" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="S17" s="6" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="T17" s="6" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="U17" s="6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="18" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1546,28 +1545,28 @@
       </c>
       <c r="M18" s="6"/>
       <c r="N18" s="6" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="O18" s="6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P18" s="6" t="s">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="Q18" s="6" t="s">
-        <v>15</v>
+        <v>37</v>
       </c>
       <c r="R18" s="6" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="S18" s="6" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="T18" s="6" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="U18" s="6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="19" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1598,28 +1597,28 @@
       </c>
       <c r="M19" s="6"/>
       <c r="N19" s="6" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="O19" s="6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P19" s="6" t="s">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="Q19" s="6" t="s">
-        <v>15</v>
+        <v>37</v>
       </c>
       <c r="R19" s="6" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="S19" s="6" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="T19" s="6" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="U19" s="6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="20" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1650,28 +1649,28 @@
       </c>
       <c r="M20" s="12"/>
       <c r="N20" s="6" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="O20" s="6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="P20" s="6" t="s">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="Q20" s="6" t="s">
-        <v>15</v>
+        <v>37</v>
       </c>
       <c r="R20" s="6" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="S20" s="6" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="T20" s="6" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="U20" s="6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="X20" s="13"/>
       <c r="Y20" s="13"/>
@@ -1965,7 +1964,7 @@
       <c r="H26" t="s">
         <v>25</v>
       </c>
-      <c r="J26" s="14" t="s">
+      <c r="J26" s="6" t="s">
         <v>23</v>
       </c>
       <c r="K26" s="6" t="s">
@@ -2021,7 +2020,7 @@
       <c r="H27" t="s">
         <v>25</v>
       </c>
-      <c r="J27" s="14"/>
+      <c r="J27" s="6"/>
       <c r="K27" s="6" t="s">
         <v>27</v>
       </c>
@@ -3141,7 +3140,7 @@
       <c r="H47" t="s">
         <v>25</v>
       </c>
-      <c r="J47" s="14" t="s">
+      <c r="J47" s="6" t="s">
         <v>23</v>
       </c>
       <c r="K47" s="6" t="s">

</xml_diff>